<commit_message>
feat(client): implement grade navigation sidebar, filter dropdown toolbar, and floating speeddial
</commit_message>
<xml_diff>
--- a/client/public/templates/قالب_کارنامه_دانش‌آموزی.xlsx
+++ b/client/public/templates/قالب_کارنامه_دانش‌آموزی.xlsx
@@ -456,7 +456,7 @@
         <v>علیرضا حسینی</v>
       </c>
       <c r="B2" t="str">
-        <v>دهم ریاضی ۱</v>
+        <v>هفتم ۱</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -494,7 +494,7 @@
         <v>محمد صادقی</v>
       </c>
       <c r="B3" t="str">
-        <v>دهم ریاضی ۱</v>
+        <v>هفتم ۱</v>
       </c>
       <c r="C3">
         <v>4</v>
@@ -532,7 +532,7 @@
         <v>سارا رحیمی</v>
       </c>
       <c r="B4" t="str">
-        <v>دهم تجربی ۲</v>
+        <v>هفتم ۲</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -570,7 +570,7 @@
         <v>امیررضا کریمی</v>
       </c>
       <c r="B5" t="str">
-        <v>دهم ریاضی ۱</v>
+        <v>هفتم ۱</v>
       </c>
       <c r="C5">
         <v>2</v>
@@ -608,7 +608,7 @@
         <v>فاطمه نوری</v>
       </c>
       <c r="B6" t="str">
-        <v>دهم تجربی ۲</v>
+        <v>هفتم ۲</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -646,7 +646,7 @@
         <v>پارسا مرادی</v>
       </c>
       <c r="B7" t="str">
-        <v>یازدهم ریاضی ۱</v>
+        <v>هفتم ۳</v>
       </c>
       <c r="C7">
         <v>6</v>

</xml_diff>